<commit_message>
Added error msg sending
</commit_message>
<xml_diff>
--- a/config/Major_brands_PS.xlsx
+++ b/config/Major_brands_PS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://atvtireinc-my.sharepoint.com/personal/vjdelrosario_avatco_com/Documents/Desktop/MWF Offers/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{5088AF8D-BBC5-4B91-9D0C-432FA8F42425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85EA9C0E-E86C-4E83-8840-C387F62D221C}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="8_{5088AF8D-BBC5-4B91-9D0C-432FA8F42425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46A69990-8714-4A37-B1FA-F812558B07CF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{77F47AA6-6586-4053-928E-5FE2A2881B5B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{77F47AA6-6586-4053-928E-5FE2A2881B5B}"/>
   </bookViews>
   <sheets>
     <sheet name="MB" sheetId="1" r:id="rId1"/>

</xml_diff>